<commit_message>
moca-t: fix drawing loading/printing, correct abstract norm coefficient, add chartNumber, implement silent cloud upload, and enhance merge_data.py
</commit_message>
<xml_diff>
--- a/reports/all_assessments_latest.xlsx
+++ b/reports/all_assessments_latest.xlsx
@@ -1,19 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="完整資料" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="摘要統計" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="風險分布" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="類型分布" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="性別_風險交叉表" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="年齡組_類型交叉表" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="教育程度_風險交叉表" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="結構問卷資料" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="問卷摘要統計" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="問卷_性別_風險交叉表" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="問卷_年齡組_類型交叉表" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1825,10 +1822,8 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>數值</t>
-        </is>
+      <c r="B1" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="2">
@@ -1986,50 +1981,77 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>風險等級</t>
+          <t>性別</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>個案數</t>
+          <t>high</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>百分比</t>
+          <t>moderate</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>總計</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>moderate</t>
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>女</t>
         </is>
       </c>
       <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>男</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C3" t="n">
         <v>2</v>
       </c>
-      <c r="C2" t="n">
-        <v>66.67</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
+      <c r="D3" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>總計</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
         <v>1</v>
       </c>
-      <c r="C3" t="n">
-        <v>33.33</v>
+      <c r="C4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4" t="n">
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -2043,147 +2065,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>失智症類型</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>個案數</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>百分比</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>PPA</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>2</v>
-      </c>
-      <c r="C2" t="n">
-        <v>66.67</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>DLB</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C3" t="n">
-        <v>33.33</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>性別</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>moderate</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>總計</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="1" t="inlineStr">
-        <is>
-          <t>女</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D2" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="1" t="inlineStr">
-        <is>
-          <t>男</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>0</v>
-      </c>
-      <c r="C3" t="n">
-        <v>2</v>
-      </c>
-      <c r="D3" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="1" t="inlineStr">
-        <is>
-          <t>總計</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>1</v>
-      </c>
-      <c r="C4" t="n">
-        <v>2</v>
-      </c>
-      <c r="D4" t="n">
-        <v>3</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
@@ -2244,88 +2125,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>教育程度</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>moderate</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>總計</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="1" t="inlineStr">
-        <is>
-          <t>不識字</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D2" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="1" t="inlineStr">
-        <is>
-          <t>大學</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>0</v>
-      </c>
-      <c r="C3" t="n">
-        <v>2</v>
-      </c>
-      <c r="D3" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="1" t="inlineStr">
-        <is>
-          <t>總計</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>1</v>
-      </c>
-      <c r="C4" t="n">
-        <v>2</v>
-      </c>
-      <c r="D4" t="n">
-        <v>3</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>